<commit_message>
Increment version to 18.0.1.0.25. Introduce bilingual bank details in invoice templates, enhancing the `res.partner.bank` model with new fields for payment instructions, bank name, address, and account details in both English and Arabic. Update invoice report views to display structured bank information, ensuring clarity for users. Add a new view for managing bank details in the Odoo interface.
</commit_message>
<xml_diff>
--- a/rgb_workover_operations/report/excel_templates/daily_report_template.xlsx
+++ b/rgb_workover_operations/report/excel_templates/daily_report_template.xlsx
@@ -204,7 +204,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="94">
+  <borders count="106">
     <border>
       <left/>
       <right/>
@@ -1422,12 +1422,148 @@
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="hair">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="double">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1933,6 +2069,26 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="84" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="98" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="99" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="101" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="99" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="102" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="100" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="99" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2315,7 +2471,7 @@
     <col width="8.14062" customWidth="1" min="11" max="11"/>
     <col width="1.57031" customWidth="1" min="12" max="12"/>
     <col width="10.1406" customWidth="1" min="13" max="13"/>
-    <col width="9.14062" customWidth="1" min="14" max="14"/>
+    <col width="0.1" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.1" customHeight="1">
@@ -2934,26 +3090,21 @@
           <t>TO</t>
         </is>
       </c>
-      <c r="C22" s="96" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="D22" s="97" t="n"/>
+      <c r="C22" s="192" t="n"/>
+      <c r="D22" s="37" t="n"/>
       <c r="E22" s="37" t="n"/>
       <c r="F22" s="37" t="n"/>
       <c r="G22" s="37" t="n"/>
       <c r="H22" s="37" t="n"/>
       <c r="I22" s="37" t="n"/>
-      <c r="J22" s="40" t="n"/>
-      <c r="K22" s="98" t="inlineStr">
+      <c r="J22" s="41" t="inlineStr">
         <is>
           <t>TIME BREAK DOWN</t>
         </is>
       </c>
+      <c r="K22" s="37" t="n"/>
       <c r="L22" s="37" t="n"/>
-      <c r="M22" s="37" t="n"/>
-      <c r="N22" s="40" t="n"/>
+      <c r="M22" s="40" t="n"/>
       <c r="P22" s="99" t="n"/>
     </row>
     <row r="23" ht="12" customHeight="1">
@@ -2963,28 +3114,27 @@
       <c r="B23" s="101" t="n">
         <v>0.75</v>
       </c>
-      <c r="C23" s="102" t="inlineStr">
+      <c r="C23" s="193" t="inlineStr">
         <is>
           <t>RIG MOVE &amp; RIG /UP</t>
         </is>
       </c>
-      <c r="D23" s="103" t="inlineStr">
-        <is>
-          <t>MOVE RIG &amp; RIG EQUIP F/G-71-91 TO D-43-H DISTANCE ONE WAY 15 KM 100%</t>
-        </is>
-      </c>
+      <c r="D23" s="104" t="n"/>
       <c r="E23" s="104" t="n"/>
       <c r="F23" s="104" t="n"/>
       <c r="G23" s="104" t="n"/>
       <c r="H23" s="104" t="n"/>
       <c r="I23" s="104" t="n"/>
-      <c r="J23" s="105" t="n"/>
-      <c r="K23" s="106" t="inlineStr">
+      <c r="J23" s="51" t="inlineStr">
         <is>
           <t>OPERATION</t>
         </is>
       </c>
-      <c r="L23" s="104" t="n"/>
+      <c r="K23" s="44" t="n"/>
+      <c r="L23" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="53" t="n"/>
       <c r="N23" s="107" t="n">
         <v>0</v>
       </c>
@@ -2992,24 +3142,22 @@
     <row r="24" ht="9.75" customHeight="1">
       <c r="A24" s="100" t="n"/>
       <c r="B24" s="101" t="n"/>
-      <c r="C24" s="108" t="n"/>
-      <c r="D24" s="103" t="inlineStr">
-        <is>
-          <t>CLEAN LEVEL LOCATION</t>
-        </is>
-      </c>
+      <c r="C24" s="195" t="n"/>
+      <c r="D24" s="104" t="n"/>
       <c r="E24" s="104" t="n"/>
       <c r="F24" s="104" t="n"/>
       <c r="G24" s="104" t="n"/>
       <c r="H24" s="104" t="n"/>
       <c r="I24" s="104" t="n"/>
-      <c r="J24" s="105" t="n"/>
-      <c r="K24" s="109" t="inlineStr">
+      <c r="J24" s="51" t="inlineStr">
         <is>
           <t>RIG MOVE &amp; RIG /UP</t>
         </is>
       </c>
-      <c r="L24" s="49" t="n"/>
+      <c r="K24" s="44" t="n"/>
+      <c r="L24" s="52" t="n">
+        <v>5</v>
+      </c>
       <c r="M24" s="53" t="n"/>
       <c r="N24" s="107" t="n">
         <v>5</v>
@@ -3020,25 +3168,23 @@
     <row r="25" ht="9.75" customHeight="1">
       <c r="A25" s="100" t="n"/>
       <c r="B25" s="101" t="n"/>
-      <c r="C25" s="108" t="n"/>
-      <c r="D25" s="103" t="inlineStr">
-        <is>
-          <t>DISCONNECT PRODCTION LINE</t>
-        </is>
-      </c>
+      <c r="C25" s="195" t="n"/>
+      <c r="D25" s="104" t="n"/>
       <c r="E25" s="104" t="n"/>
       <c r="F25" s="104" t="n"/>
       <c r="G25" s="104" t="n"/>
       <c r="H25" s="104" t="n"/>
       <c r="I25" s="104" t="n"/>
-      <c r="J25" s="105" t="n"/>
-      <c r="K25" s="112" t="inlineStr">
+      <c r="J25" s="51" t="inlineStr">
         <is>
           <t>STANDBY W/CREW</t>
         </is>
       </c>
-      <c r="L25" s="22" t="n"/>
-      <c r="M25" s="27" t="n"/>
+      <c r="K25" s="44" t="n"/>
+      <c r="L25" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="53" t="n"/>
       <c r="N25" s="107" t="n">
         <v>0</v>
       </c>
@@ -3046,25 +3192,23 @@
     <row r="26" ht="10.5" customHeight="1">
       <c r="A26" s="100" t="n"/>
       <c r="B26" s="101" t="n"/>
-      <c r="C26" s="108" t="n"/>
-      <c r="D26" s="103" t="inlineStr">
-        <is>
-          <t>SPOT RIG &amp; RIG EQUIP INSIDE LOC 40%</t>
-        </is>
-      </c>
+      <c r="C26" s="195" t="n"/>
+      <c r="D26" s="104" t="n"/>
       <c r="E26" s="104" t="n"/>
       <c r="F26" s="104" t="n"/>
       <c r="G26" s="104" t="n"/>
       <c r="H26" s="104" t="n"/>
       <c r="I26" s="104" t="n"/>
-      <c r="J26" s="105" t="n"/>
-      <c r="K26" s="112" t="inlineStr">
+      <c r="J26" s="51" t="inlineStr">
         <is>
           <t>DOWN TIME</t>
         </is>
       </c>
-      <c r="L26" s="22" t="n"/>
-      <c r="M26" s="27" t="n"/>
+      <c r="K26" s="44" t="n"/>
+      <c r="L26" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="53" t="n"/>
       <c r="N26" s="107" t="n">
         <v>0</v>
       </c>
@@ -3072,21 +3216,23 @@
     <row r="27" ht="9.75" customHeight="1">
       <c r="A27" s="100" t="n"/>
       <c r="B27" s="101" t="n"/>
-      <c r="C27" s="108" t="n"/>
-      <c r="D27" s="103" t="n"/>
+      <c r="C27" s="195" t="n"/>
+      <c r="D27" s="104" t="n"/>
       <c r="E27" s="104" t="n"/>
       <c r="F27" s="104" t="n"/>
       <c r="G27" s="104" t="n"/>
       <c r="H27" s="104" t="n"/>
       <c r="I27" s="104" t="n"/>
-      <c r="J27" s="105" t="n"/>
-      <c r="K27" s="112" t="inlineStr">
+      <c r="J27" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">SHUT DOWN </t>
         </is>
       </c>
-      <c r="L27" s="22" t="n"/>
-      <c r="M27" s="27" t="n"/>
+      <c r="K27" s="44" t="n"/>
+      <c r="L27" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="53" t="n"/>
       <c r="N27" s="107" t="n">
         <v>0</v>
       </c>
@@ -3095,21 +3241,23 @@
     <row r="28" ht="9.75" customHeight="1">
       <c r="A28" s="100" t="n"/>
       <c r="B28" s="101" t="n"/>
-      <c r="C28" s="108" t="n"/>
-      <c r="D28" s="103" t="n"/>
+      <c r="C28" s="195" t="n"/>
+      <c r="D28" s="104" t="n"/>
       <c r="E28" s="104" t="n"/>
       <c r="F28" s="104" t="n"/>
       <c r="G28" s="104" t="n"/>
       <c r="H28" s="104" t="n"/>
       <c r="I28" s="104" t="n"/>
-      <c r="J28" s="105" t="n"/>
-      <c r="K28" s="112" t="inlineStr">
+      <c r="J28" s="51" t="inlineStr">
         <is>
           <t>REPAIR</t>
         </is>
       </c>
-      <c r="L28" s="22" t="n"/>
-      <c r="M28" s="27" t="n"/>
+      <c r="K28" s="44" t="n"/>
+      <c r="L28" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="53" t="n"/>
       <c r="N28" s="107" t="n">
         <v>0</v>
       </c>
@@ -3117,17 +3265,19 @@
     <row r="29" ht="10.5" customHeight="1">
       <c r="A29" s="100" t="n"/>
       <c r="B29" s="101" t="n"/>
-      <c r="C29" s="108" t="n"/>
-      <c r="D29" s="103" t="n"/>
+      <c r="C29" s="195" t="n"/>
+      <c r="D29" s="104" t="n"/>
       <c r="E29" s="104" t="n"/>
       <c r="F29" s="104" t="n"/>
       <c r="G29" s="104" t="n"/>
       <c r="H29" s="104" t="n"/>
       <c r="I29" s="104" t="n"/>
-      <c r="J29" s="105" t="n"/>
-      <c r="K29" s="114" t="n"/>
-      <c r="L29" s="22" t="n"/>
-      <c r="M29" s="27" t="n"/>
+      <c r="J29" s="51" t="n"/>
+      <c r="K29" s="44" t="n"/>
+      <c r="L29" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="53" t="n"/>
       <c r="N29" s="107" t="n">
         <v>0</v>
       </c>
@@ -3136,21 +3286,24 @@
     <row r="30" ht="12.95" customHeight="1">
       <c r="A30" s="100" t="n"/>
       <c r="B30" s="101" t="n"/>
-      <c r="C30" s="108" t="n"/>
-      <c r="D30" s="116" t="n"/>
+      <c r="C30" s="195" t="n"/>
+      <c r="D30" s="104" t="n"/>
       <c r="E30" s="104" t="n"/>
       <c r="F30" s="104" t="n"/>
       <c r="G30" s="104" t="n"/>
       <c r="H30" s="104" t="n"/>
       <c r="I30" s="104" t="n"/>
-      <c r="J30" s="105" t="n"/>
-      <c r="K30" s="117" t="n"/>
-      <c r="L30" s="118" t="inlineStr">
+      <c r="J30" s="51" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="M30" s="29" t="n"/>
+      <c r="K30" s="44" t="n"/>
+      <c r="L30" s="52">
+        <f>SUM(L23:L29)</f>
+        <v/>
+      </c>
+      <c r="M30" s="53" t="n"/>
       <c r="N30" s="119">
         <f>SUM(N23:N29)</f>
         <v/>
@@ -3159,14 +3312,13 @@
     <row r="31" ht="12.95" customHeight="1">
       <c r="A31" s="100" t="n"/>
       <c r="B31" s="101" t="n"/>
-      <c r="C31" s="108" t="n"/>
-      <c r="D31" s="116" t="n"/>
+      <c r="C31" s="195" t="n"/>
+      <c r="D31" s="104" t="n"/>
       <c r="E31" s="104" t="n"/>
       <c r="F31" s="104" t="n"/>
       <c r="G31" s="104" t="n"/>
       <c r="H31" s="104" t="n"/>
       <c r="I31" s="104" t="n"/>
-      <c r="J31" s="105" t="n"/>
       <c r="K31" s="120" t="n"/>
       <c r="L31" s="37" t="n"/>
       <c r="M31" s="37" t="n"/>
@@ -3175,14 +3327,13 @@
     <row r="32" ht="12.95" customHeight="1">
       <c r="A32" s="121" t="n"/>
       <c r="B32" s="108" t="n"/>
-      <c r="C32" s="108" t="n"/>
-      <c r="D32" s="116" t="n"/>
+      <c r="C32" s="195" t="n"/>
+      <c r="D32" s="104" t="n"/>
       <c r="E32" s="104" t="n"/>
       <c r="F32" s="104" t="n"/>
       <c r="G32" s="104" t="n"/>
       <c r="H32" s="104" t="n"/>
       <c r="I32" s="104" t="n"/>
-      <c r="J32" s="105" t="n"/>
       <c r="K32" s="122" t="n"/>
       <c r="L32" s="123" t="inlineStr">
         <is>
@@ -3199,14 +3350,13 @@
     <row r="33" ht="12" customHeight="1">
       <c r="A33" s="121" t="n"/>
       <c r="B33" s="125" t="n"/>
-      <c r="C33" s="126" t="n"/>
-      <c r="D33" s="127" t="n"/>
+      <c r="C33" s="198" t="n"/>
+      <c r="D33" s="104" t="n"/>
       <c r="E33" s="104" t="n"/>
       <c r="F33" s="104" t="n"/>
       <c r="G33" s="104" t="n"/>
       <c r="H33" s="104" t="n"/>
       <c r="I33" s="104" t="n"/>
-      <c r="J33" s="105" t="n"/>
       <c r="K33" s="128" t="inlineStr">
         <is>
           <t>OXY</t>
@@ -3223,14 +3373,13 @@
     <row r="34" ht="11.25" customHeight="1">
       <c r="A34" s="131" t="n"/>
       <c r="B34" s="108" t="n"/>
-      <c r="C34" s="108" t="n"/>
-      <c r="D34" s="132" t="n"/>
+      <c r="C34" s="195" t="n"/>
+      <c r="D34" s="104" t="n"/>
       <c r="E34" s="104" t="n"/>
       <c r="F34" s="104" t="n"/>
       <c r="G34" s="104" t="n"/>
       <c r="H34" s="104" t="n"/>
       <c r="I34" s="104" t="n"/>
-      <c r="J34" s="105" t="n"/>
       <c r="K34" s="94" t="inlineStr">
         <is>
           <t>ACYT</t>
@@ -3247,14 +3396,13 @@
     <row r="35" ht="12.95" customHeight="1">
       <c r="A35" s="131" t="n"/>
       <c r="B35" s="108" t="n"/>
-      <c r="C35" s="108" t="n"/>
-      <c r="D35" s="132" t="n"/>
+      <c r="C35" s="195" t="n"/>
+      <c r="D35" s="104" t="n"/>
       <c r="E35" s="104" t="n"/>
       <c r="F35" s="104" t="n"/>
       <c r="G35" s="104" t="n"/>
       <c r="H35" s="104" t="n"/>
       <c r="I35" s="104" t="n"/>
-      <c r="J35" s="105" t="n"/>
       <c r="K35" s="133" t="inlineStr">
         <is>
           <t>ENGINE OIL 40wt</t>
@@ -3269,14 +3417,13 @@
     <row r="36" ht="12.95" customHeight="1">
       <c r="A36" s="131" t="n"/>
       <c r="B36" s="108" t="n"/>
-      <c r="C36" s="108" t="n"/>
-      <c r="D36" s="135" t="n"/>
+      <c r="C36" s="195" t="n"/>
+      <c r="D36" s="104" t="n"/>
       <c r="E36" s="104" t="n"/>
       <c r="F36" s="104" t="n"/>
       <c r="G36" s="104" t="n"/>
       <c r="H36" s="104" t="n"/>
       <c r="I36" s="104" t="n"/>
-      <c r="J36" s="105" t="n"/>
       <c r="K36" s="136" t="inlineStr">
         <is>
           <t xml:space="preserve">HYDRAULIC 37wt. </t>
@@ -3293,14 +3440,13 @@
     <row r="37" ht="12.95" customHeight="1">
       <c r="A37" s="100" t="n"/>
       <c r="B37" s="108" t="n"/>
-      <c r="C37" s="108" t="n"/>
-      <c r="D37" s="135" t="n"/>
+      <c r="C37" s="195" t="n"/>
+      <c r="D37" s="104" t="n"/>
       <c r="E37" s="104" t="n"/>
       <c r="F37" s="104" t="n"/>
       <c r="G37" s="104" t="n"/>
       <c r="H37" s="104" t="n"/>
       <c r="I37" s="104" t="n"/>
-      <c r="J37" s="105" t="n"/>
       <c r="K37" s="136" t="inlineStr">
         <is>
           <t>GEAR 90wt</t>
@@ -3322,14 +3468,13 @@
     <row r="38" ht="12.95" customHeight="1">
       <c r="A38" s="131" t="n"/>
       <c r="B38" s="138" t="n"/>
-      <c r="C38" s="138" t="n"/>
-      <c r="D38" s="139" t="n"/>
+      <c r="C38" s="199" t="n"/>
+      <c r="D38" s="104" t="n"/>
       <c r="E38" s="104" t="n"/>
       <c r="F38" s="104" t="n"/>
       <c r="G38" s="104" t="n"/>
       <c r="H38" s="104" t="n"/>
       <c r="I38" s="104" t="n"/>
-      <c r="J38" s="105" t="n"/>
       <c r="K38" s="136" t="inlineStr">
         <is>
           <t>A.T.F</t>
@@ -3344,14 +3489,13 @@
     <row r="39" ht="12.95" customHeight="1">
       <c r="A39" s="131" t="n"/>
       <c r="B39" s="138" t="n"/>
-      <c r="C39" s="138" t="n"/>
-      <c r="D39" s="135" t="n"/>
+      <c r="C39" s="199" t="n"/>
+      <c r="D39" s="104" t="n"/>
       <c r="E39" s="104" t="n"/>
       <c r="F39" s="104" t="n"/>
       <c r="G39" s="104" t="n"/>
       <c r="H39" s="104" t="n"/>
       <c r="I39" s="104" t="n"/>
-      <c r="J39" s="105" t="n"/>
       <c r="K39" s="136" t="inlineStr">
         <is>
           <t xml:space="preserve">GREASE    </t>
@@ -3368,7 +3512,13 @@
     <row r="40" ht="12.95" customHeight="1">
       <c r="A40" s="131" t="n"/>
       <c r="B40" s="138" t="n"/>
-      <c r="C40" s="138" t="n"/>
+      <c r="C40" s="199" t="n"/>
+      <c r="D40" s="104" t="n"/>
+      <c r="E40" s="104" t="n"/>
+      <c r="F40" s="104" t="n"/>
+      <c r="G40" s="104" t="n"/>
+      <c r="H40" s="104" t="n"/>
+      <c r="I40" s="104" t="n"/>
       <c r="K40" s="140" t="inlineStr">
         <is>
           <t>DIESEL</t>
@@ -3384,14 +3534,13 @@
     <row r="41" ht="12.95" customHeight="1">
       <c r="A41" s="131" t="n"/>
       <c r="B41" s="138" t="n"/>
-      <c r="C41" s="138" t="n"/>
-      <c r="D41" s="145" t="n"/>
+      <c r="C41" s="199" t="n"/>
+      <c r="D41" s="104" t="n"/>
       <c r="E41" s="104" t="n"/>
       <c r="F41" s="104" t="n"/>
       <c r="G41" s="104" t="n"/>
       <c r="H41" s="104" t="n"/>
       <c r="I41" s="104" t="n"/>
-      <c r="J41" s="105" t="n"/>
       <c r="K41" s="146" t="inlineStr">
         <is>
           <t>DRILLING LINE &amp; TON MILS</t>
@@ -3404,14 +3553,13 @@
     <row r="42" ht="12.95" customHeight="1">
       <c r="A42" s="131" t="n"/>
       <c r="B42" s="138" t="n"/>
-      <c r="C42" s="138" t="n"/>
-      <c r="D42" s="147" t="n"/>
+      <c r="C42" s="199" t="n"/>
+      <c r="D42" s="104" t="n"/>
       <c r="E42" s="104" t="n"/>
       <c r="F42" s="104" t="n"/>
       <c r="G42" s="104" t="n"/>
       <c r="H42" s="104" t="n"/>
       <c r="I42" s="104" t="n"/>
-      <c r="J42" s="105" t="n"/>
       <c r="K42" s="148" t="inlineStr">
         <is>
           <t>DRILLING LINE &amp; TON MILS</t>
@@ -3426,14 +3574,13 @@
     <row r="43" ht="12.95" customHeight="1">
       <c r="A43" s="131" t="n"/>
       <c r="B43" s="138" t="n"/>
-      <c r="C43" s="138" t="n"/>
-      <c r="D43" s="150" t="n"/>
+      <c r="C43" s="199" t="n"/>
+      <c r="D43" s="104" t="n"/>
       <c r="E43" s="104" t="n"/>
       <c r="F43" s="104" t="n"/>
       <c r="G43" s="104" t="n"/>
       <c r="H43" s="104" t="n"/>
       <c r="I43" s="104" t="n"/>
-      <c r="J43" s="105" t="n"/>
       <c r="K43" s="151" t="inlineStr">
         <is>
           <t xml:space="preserve">DRILLING LINE LENGTH </t>
@@ -3448,14 +3595,13 @@
     <row r="44" ht="12.95" customHeight="1">
       <c r="A44" s="131" t="n"/>
       <c r="B44" s="138" t="n"/>
-      <c r="C44" s="138" t="n"/>
-      <c r="D44" s="145" t="n"/>
+      <c r="C44" s="199" t="n"/>
+      <c r="D44" s="104" t="n"/>
       <c r="E44" s="104" t="n"/>
       <c r="F44" s="104" t="n"/>
       <c r="G44" s="104" t="n"/>
       <c r="H44" s="104" t="n"/>
       <c r="I44" s="104" t="n"/>
-      <c r="J44" s="105" t="n"/>
       <c r="K44" s="153" t="inlineStr">
         <is>
           <t>DRILLING LINE SLIP</t>
@@ -3471,14 +3617,13 @@
     <row r="45" ht="12.95" customHeight="1">
       <c r="A45" s="156" t="n"/>
       <c r="B45" s="138" t="n"/>
-      <c r="C45" s="138" t="n"/>
-      <c r="D45" s="157" t="n"/>
-      <c r="E45" s="158" t="n"/>
-      <c r="F45" s="158" t="n"/>
-      <c r="G45" s="158" t="n"/>
-      <c r="H45" s="158" t="n"/>
-      <c r="I45" s="158" t="n"/>
-      <c r="J45" s="159" t="n"/>
+      <c r="C45" s="199" t="n"/>
+      <c r="D45" s="104" t="n"/>
+      <c r="E45" s="104" t="n"/>
+      <c r="F45" s="104" t="n"/>
+      <c r="G45" s="104" t="n"/>
+      <c r="H45" s="104" t="n"/>
+      <c r="I45" s="104" t="n"/>
       <c r="K45" s="160" t="inlineStr">
         <is>
           <t>DRILLING LINE TOTAL CUT</t>
@@ -3828,17 +3973,19 @@
       <c r="M57" s="7" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="180">
+  <mergeCells count="189">
+    <mergeCell ref="C36:I36"/>
     <mergeCell ref="E3:I3"/>
     <mergeCell ref="M43:N43"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="J19:K19"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="L19:M19"/>
-    <mergeCell ref="D24:J24"/>
+    <mergeCell ref="J28:K28"/>
     <mergeCell ref="K56:M56"/>
-    <mergeCell ref="D33:J33"/>
+    <mergeCell ref="L28:M28"/>
     <mergeCell ref="B12:C12"/>
+    <mergeCell ref="C28:I28"/>
     <mergeCell ref="K35:L35"/>
     <mergeCell ref="E51:F51"/>
     <mergeCell ref="A54:B54"/>
@@ -3847,46 +3994,43 @@
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C54:D54"/>
     <mergeCell ref="J17:M17"/>
-    <mergeCell ref="D26:J26"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="D35:J35"/>
     <mergeCell ref="C50:D50"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="A1:C6"/>
+    <mergeCell ref="C30:I30"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="L14:M14"/>
     <mergeCell ref="A56:B56"/>
     <mergeCell ref="C56:D56"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="C45:I45"/>
     <mergeCell ref="C21:G21"/>
+    <mergeCell ref="L29:M29"/>
     <mergeCell ref="K42:L42"/>
     <mergeCell ref="M36:N36"/>
     <mergeCell ref="M33:N33"/>
     <mergeCell ref="M45:N45"/>
     <mergeCell ref="I52:J52"/>
-    <mergeCell ref="K25:M25"/>
     <mergeCell ref="A53:B53"/>
+    <mergeCell ref="C31:I31"/>
     <mergeCell ref="J21:K21"/>
+    <mergeCell ref="C40:I40"/>
     <mergeCell ref="L21:M21"/>
     <mergeCell ref="K37:L37"/>
     <mergeCell ref="E53:F53"/>
+    <mergeCell ref="J23:K23"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="K29:M29"/>
-    <mergeCell ref="D37:J37"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C23:I23"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="E55:F55"/>
     <mergeCell ref="L16:M16"/>
-    <mergeCell ref="D39:J39"/>
     <mergeCell ref="M44:N44"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="E48:F48"/>
-    <mergeCell ref="D29:J29"/>
-    <mergeCell ref="D23:J23"/>
-    <mergeCell ref="D38:J38"/>
     <mergeCell ref="C20:G20"/>
     <mergeCell ref="C47:D47"/>
     <mergeCell ref="I54:J54"/>
@@ -3894,6 +4038,9 @@
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="I7:J7"/>
     <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C34:I34"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="C42:I42"/>
     <mergeCell ref="K7:M7"/>
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="I56:J56"/>
@@ -3904,58 +4051,67 @@
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="K43:L43"/>
     <mergeCell ref="L20:M20"/>
+    <mergeCell ref="C29:I29"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="D27:J27"/>
+    <mergeCell ref="K41:N41"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="K41:N41"/>
+    <mergeCell ref="C44:I44"/>
+    <mergeCell ref="C22:I22"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="C53:D53"/>
     <mergeCell ref="J48:K48"/>
     <mergeCell ref="L48:M48"/>
-    <mergeCell ref="D28:J28"/>
     <mergeCell ref="E50:F50"/>
+    <mergeCell ref="J22:M22"/>
+    <mergeCell ref="J29:K29"/>
     <mergeCell ref="M34:N34"/>
     <mergeCell ref="G11:H11"/>
-    <mergeCell ref="D25:J25"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="I49:M49"/>
-    <mergeCell ref="D30:J30"/>
+    <mergeCell ref="E52:F52"/>
     <mergeCell ref="K45:L45"/>
-    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="C32:I32"/>
     <mergeCell ref="M39:N39"/>
+    <mergeCell ref="C38:I38"/>
     <mergeCell ref="L47:M47"/>
     <mergeCell ref="E46:M46"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="L24:M24"/>
     <mergeCell ref="D4:G5"/>
     <mergeCell ref="L18:M18"/>
     <mergeCell ref="K44:L44"/>
+    <mergeCell ref="C24:I24"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="L8:M8"/>
+    <mergeCell ref="C33:I33"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="M40:N40"/>
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="D31:J31"/>
+    <mergeCell ref="J26:K26"/>
     <mergeCell ref="G47:I47"/>
+    <mergeCell ref="L26:M26"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C46:D46"/>
+    <mergeCell ref="C26:I26"/>
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="J16:K16"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="M37:N37"/>
     <mergeCell ref="C51:D51"/>
     <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="C35:I35"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="L25:M25"/>
     <mergeCell ref="C48:D48"/>
+    <mergeCell ref="C25:I25"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="K31:N31"/>
-    <mergeCell ref="D32:J32"/>
-    <mergeCell ref="K24:M24"/>
     <mergeCell ref="G51:H51"/>
     <mergeCell ref="I51:J51"/>
-    <mergeCell ref="D41:J41"/>
     <mergeCell ref="E54:F54"/>
     <mergeCell ref="G54:H54"/>
     <mergeCell ref="M38:N38"/>
@@ -3963,51 +4119,49 @@
     <mergeCell ref="G50:H50"/>
     <mergeCell ref="H9:J9"/>
     <mergeCell ref="I50:J50"/>
-    <mergeCell ref="K26:M26"/>
     <mergeCell ref="K51:M51"/>
-    <mergeCell ref="D43:J43"/>
     <mergeCell ref="E56:F56"/>
     <mergeCell ref="G56:H56"/>
     <mergeCell ref="K50:M50"/>
     <mergeCell ref="G52:H52"/>
+    <mergeCell ref="C39:I39"/>
     <mergeCell ref="J14:K14"/>
-    <mergeCell ref="D42:J42"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="K36:L36"/>
     <mergeCell ref="K52:M52"/>
     <mergeCell ref="L13:M13"/>
-    <mergeCell ref="D44:J44"/>
+    <mergeCell ref="C37:I37"/>
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="J15:K15"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="L15:M15"/>
     <mergeCell ref="C55:D55"/>
-    <mergeCell ref="D34:J34"/>
     <mergeCell ref="G53:H53"/>
     <mergeCell ref="I53:J53"/>
+    <mergeCell ref="L23:M23"/>
     <mergeCell ref="K53:M53"/>
     <mergeCell ref="A50:B50"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="D22:J22"/>
-    <mergeCell ref="D36:J36"/>
-    <mergeCell ref="K28:M28"/>
     <mergeCell ref="I55:J55"/>
-    <mergeCell ref="D45:J45"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="M42:N42"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="K39:L39"/>
     <mergeCell ref="J47:K47"/>
+    <mergeCell ref="C41:I41"/>
     <mergeCell ref="G55:H55"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="K22:N22"/>
     <mergeCell ref="K38:L38"/>
     <mergeCell ref="M32:N32"/>
     <mergeCell ref="K54:M54"/>
+    <mergeCell ref="C43:I43"/>
     <mergeCell ref="J18:K18"/>
     <mergeCell ref="K55:M55"/>
     <mergeCell ref="G48:I48"/>
+    <mergeCell ref="L27:M27"/>
     <mergeCell ref="D1:J2"/>
+    <mergeCell ref="C27:I27"/>
     <mergeCell ref="E47:F47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>